<commit_message>
done till internal audit stratgeies form submission. Report Left
</commit_message>
<xml_diff>
--- a/Audit_Code/public/internal_audit_sheet.xlsx
+++ b/Audit_Code/public/internal_audit_sheet.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="18">
   <si>
     <t>L1 Number</t>
   </si>
@@ -38,9 +38,6 @@
     <t>L2 Text</t>
   </si>
   <si>
-    <t>Planning and Risk Assessment</t>
-  </si>
-  <si>
     <t>Understand the Business</t>
   </si>
   <si>
@@ -60,6 +57,27 @@
   </si>
   <si>
     <t>Develop Audit Procedures</t>
+  </si>
+  <si>
+    <t>Internal Audit Strategy</t>
+  </si>
+  <si>
+    <t>Risk Based Audit Plan (RBAP)</t>
+  </si>
+  <si>
+    <t>Risk Assessment for the Purpose of Internal Audit</t>
+  </si>
+  <si>
+    <t>Audit Sampling Policies/Methodoligies/Processes</t>
+  </si>
+  <si>
+    <t>Audit Results and Reporting</t>
+  </si>
+  <si>
+    <t>Follow up of Audit Report/Recommendations</t>
+  </si>
+  <si>
+    <t>Record Keeping of Audit Reports and Working Papers</t>
   </si>
 </sst>
 </file>
@@ -386,10 +404,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="21.21875" customWidth="1"/>
+    <col min="2" max="2" width="50.21875" customWidth="1"/>
     <col min="3" max="3" width="10.21875" customWidth="1"/>
     <col min="4" max="4" width="34.109375" customWidth="1"/>
   </cols>
@@ -413,13 +431,13 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2" t="s">
         <v>4</v>
-      </c>
-      <c r="C2">
-        <v>1</v>
-      </c>
-      <c r="D2" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
@@ -427,13 +445,13 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="C3">
         <v>2</v>
       </c>
       <c r="D3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
@@ -441,13 +459,13 @@
         <v>1</v>
       </c>
       <c r="B4" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="C4">
         <v>3</v>
       </c>
       <c r="D4" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
@@ -455,13 +473,13 @@
         <v>1</v>
       </c>
       <c r="B5" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="C5">
         <v>4</v>
       </c>
       <c r="D5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
@@ -469,13 +487,13 @@
         <v>1</v>
       </c>
       <c r="B6" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="C6">
         <v>5</v>
       </c>
       <c r="D6" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
@@ -483,13 +501,13 @@
         <v>1</v>
       </c>
       <c r="B7" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="C7">
         <v>6</v>
       </c>
       <c r="D7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
@@ -497,13 +515,61 @@
         <v>1</v>
       </c>
       <c r="B8" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="C8">
         <v>7</v>
       </c>
       <c r="D8" t="s">
-        <v>11</v>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>2</v>
+      </c>
+      <c r="B9" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A10">
+        <v>3</v>
+      </c>
+      <c r="B10" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A11">
+        <v>4</v>
+      </c>
+      <c r="B11" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A12">
+        <v>5</v>
+      </c>
+      <c r="B12" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A13">
+        <v>6</v>
+      </c>
+      <c r="B13" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A14">
+        <v>7</v>
+      </c>
+      <c r="B14" t="s">
+        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>